<commit_message>
chore: update performance calculations
</commit_message>
<xml_diff>
--- a/docs/Расчёты.xlsx
+++ b/docs/Расчёты.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Programming\rsschool\react-performance\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7B257B00-8D0B-4B30-8C09-F8BE79356736}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{529D0642-A9F5-423E-B68E-24D5BFC6B42C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1875" yWindow="2445" windowWidth="16200" windowHeight="9307" xr2:uid="{7A107E4D-BF9D-45CD-9CCA-4EA53CC16E3F}"/>
   </bookViews>
@@ -22,10 +22,6 @@
     </ext>
   </extLst>
 </workbook>
-</file>
-
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -388,11 +384,11 @@
         <v>96</v>
       </c>
       <c r="B1" s="1">
-        <v>49</v>
+        <v>5</v>
       </c>
       <c r="C1" s="1">
         <f>(A1-B1)/A1*100</f>
-        <v>48.958333333333329</v>
+        <v>94.791666666666657</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.45">
@@ -438,11 +434,11 @@
       </c>
       <c r="B5" s="1">
         <f>AVERAGE(B1:B4)</f>
-        <v>22.274999999999999</v>
+        <v>11.275</v>
       </c>
       <c r="C5" s="1">
         <f>AVERAGE(C1:C4)</f>
-        <v>76.873206013174496</v>
+        <v>88.331539346507824</v>
       </c>
     </row>
   </sheetData>

</xml_diff>